<commit_message>
feat: Back-end completo e front-end sendo alimentado pela nossa API
</commit_message>
<xml_diff>
--- a/DOCS/burndown2.xlsx
+++ b/DOCS/burndown2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\FATEC\sem3\API-3\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C551592-F7AB-4014-B7B3-4B725F3D6D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C38BB0C2-56FA-4643-A250-BFC4FDDDE9E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Burn1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Total de horas</t>
   </si>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t>T-22</t>
+  </si>
+  <si>
+    <t>T-23</t>
+  </si>
+  <si>
+    <t>T-24</t>
   </si>
 </sst>
 </file>
@@ -756,7 +762,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -920,67 +926,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>58</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>54</c:v>
+                  <c:v>44</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>48</c:v>
+                  <c:v>38</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45.5</c:v>
+                  <c:v>35.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45.5</c:v>
+                  <c:v>35.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>44.5</c:v>
+                  <c:v>34.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>43.5</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>43.5</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>43.5</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>43.5</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>40.5</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>40.5</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>40.5</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>40.5</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>40.5</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>40.5</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>40.5</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>40.5</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>40.5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>40.5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>40.5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1094,64 +1100,64 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>58</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>55.1</c:v>
+                  <c:v>45.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>52.2</c:v>
+                  <c:v>43.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>49.3</c:v>
+                  <c:v>40.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46.4</c:v>
+                  <c:v>38.4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>43.5</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>40.6</c:v>
+                  <c:v>33.6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>37.700000000000003</c:v>
+                  <c:v>31.2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>34.799999999999997</c:v>
+                  <c:v>28.8</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>31.900000000000002</c:v>
+                  <c:v>26.400000000000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>29</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>26.1</c:v>
+                  <c:v>21.6</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>23.200000000000003</c:v>
+                  <c:v>19.200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>20.300000000000004</c:v>
+                  <c:v>16.8</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>17.399999999999999</c:v>
+                  <c:v>14.399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>14.5</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>11.600000000000001</c:v>
+                  <c:v>9.6000000000000014</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.7000000000000028</c:v>
+                  <c:v>7.2000000000000028</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5.8000000000000043</c:v>
+                  <c:v>4.8000000000000043</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.8999999999999986</c:v>
+                  <c:v>2.3999999999999986</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -1399,7 +1405,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1563,67 +1569,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>58</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>54</c:v>
+                  <c:v>44</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>48</c:v>
+                  <c:v>38</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45.5</c:v>
+                  <c:v>35.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45.5</c:v>
+                  <c:v>35.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>44.5</c:v>
+                  <c:v>34.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>43.5</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>43.5</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>43.5</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>43.5</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>40.5</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>40.5</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>40.5</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>40.5</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>40.5</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>40.5</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>40.5</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>40.5</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>40.5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>40.5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>40.5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1737,64 +1743,64 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>58</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>55.1</c:v>
+                  <c:v>45.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>52.2</c:v>
+                  <c:v>43.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>49.3</c:v>
+                  <c:v>40.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46.4</c:v>
+                  <c:v>38.4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>43.5</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>40.6</c:v>
+                  <c:v>33.6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>37.700000000000003</c:v>
+                  <c:v>31.2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>34.799999999999997</c:v>
+                  <c:v>28.8</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>31.900000000000002</c:v>
+                  <c:v>26.400000000000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>29</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>26.1</c:v>
+                  <c:v>21.6</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>23.200000000000003</c:v>
+                  <c:v>19.200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>20.300000000000004</c:v>
+                  <c:v>16.8</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>17.399999999999999</c:v>
+                  <c:v>14.399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>14.5</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>11.600000000000001</c:v>
+                  <c:v>9.6000000000000014</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.7000000000000028</c:v>
+                  <c:v>7.2000000000000028</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5.8000000000000043</c:v>
+                  <c:v>4.8000000000000043</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.8999999999999986</c:v>
+                  <c:v>2.3999999999999986</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -2043,10 +2049,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>357867</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>144915</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>5089</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>86118</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6191250" cy="3638551"/>
     <xdr:graphicFrame macro="">
@@ -2519,7 +2525,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2543,7 +2549,7 @@
       <c r="V2" s="1"/>
       <c r="W2" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
@@ -2599,21 +2605,29 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1">
-        <v>3</v>
-      </c>
-      <c r="M4" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="M4" s="1">
+        <v>2</v>
+      </c>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
+      <c r="P4" s="1">
+        <v>2</v>
+      </c>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="1"/>
-      <c r="T4" s="1"/>
+      <c r="S4" s="1">
+        <v>2</v>
+      </c>
+      <c r="T4" s="1">
+        <v>2</v>
+      </c>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -2637,7 +2651,9 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="M5" s="1">
+        <v>2</v>
+      </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
@@ -2649,7 +2665,7 @@
       <c r="V5" s="1"/>
       <c r="W5" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
@@ -2657,7 +2673,7 @@
         <v>29</v>
       </c>
       <c r="B6" s="1">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -2669,7 +2685,9 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
+      <c r="K6" s="1">
+        <v>2.5</v>
+      </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
@@ -2683,7 +2701,7 @@
       <c r="V6" s="1"/>
       <c r="W6" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
-        <v>9.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
@@ -2706,7 +2724,9 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
+      <c r="P7" s="1">
+        <v>2</v>
+      </c>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -2715,7 +2735,7 @@
       <c r="V7" s="1"/>
       <c r="W7" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
@@ -2723,7 +2743,7 @@
         <v>31</v>
       </c>
       <c r="B8" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
@@ -2742,8 +2762,12 @@
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
+      <c r="P8" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>1</v>
+      </c>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
@@ -2751,7 +2775,7 @@
       <c r="V8" s="1"/>
       <c r="W8" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
@@ -2759,7 +2783,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -2778,17 +2802,23 @@
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
-      <c r="T9" s="1"/>
+      <c r="T9" s="1">
+        <v>1</v>
+      </c>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="1"/>
+      <c r="A10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="1">
+        <v>5</v>
+      </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -2799,14 +2829,20 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
+      <c r="M10" s="1">
+        <v>2</v>
+      </c>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
+      <c r="P10" s="1">
+        <v>2</v>
+      </c>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
-      <c r="T10" s="1"/>
+      <c r="T10" s="1">
+        <v>1</v>
+      </c>
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1">
@@ -2815,8 +2851,12 @@
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="1"/>
+      <c r="A11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="1">
+        <v>2</v>
+      </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -2830,8 +2870,12 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
+      <c r="P11" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>1</v>
+      </c>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
@@ -2960,87 +3004,87 @@
       </c>
       <c r="B16" s="9">
         <f>SUM(B2:B15)</f>
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="C16" s="6">
-        <f>B16-SUM(C2:C15)</f>
-        <v>54</v>
+        <f t="shared" ref="C16:V16" si="0">B16-SUM(C2:C15)</f>
+        <v>44</v>
       </c>
       <c r="D16" s="6">
-        <f>C16-SUM(D2:D15)</f>
-        <v>48</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
       <c r="E16" s="6">
-        <f>D16-SUM(E2:E15)</f>
-        <v>45.5</v>
+        <f t="shared" si="0"/>
+        <v>35.5</v>
       </c>
       <c r="F16" s="6">
-        <f>E16-SUM(F2:F15)</f>
-        <v>45.5</v>
+        <f t="shared" si="0"/>
+        <v>35.5</v>
       </c>
       <c r="G16" s="6">
-        <f>F16-SUM(G2:G15)</f>
-        <v>44.5</v>
+        <f t="shared" si="0"/>
+        <v>34.5</v>
       </c>
       <c r="H16" s="6">
-        <f>G16-SUM(H2:H15)</f>
-        <v>43.5</v>
+        <f t="shared" si="0"/>
+        <v>33.5</v>
       </c>
       <c r="I16" s="9">
-        <f>H16-SUM(I2:I15)</f>
-        <v>43.5</v>
+        <f t="shared" si="0"/>
+        <v>33.5</v>
       </c>
       <c r="J16" s="6">
-        <f>I16-SUM(J2:J15)</f>
-        <v>43.5</v>
+        <f t="shared" si="0"/>
+        <v>33.5</v>
       </c>
       <c r="K16" s="6">
-        <f>J16-SUM(K2:K15)</f>
-        <v>43.5</v>
+        <f t="shared" si="0"/>
+        <v>31</v>
       </c>
       <c r="L16" s="9">
-        <f>K16-SUM(L2:L15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="M16" s="6">
         <f>L16-SUM(M2:M15)</f>
-        <v>40.5</v>
+        <v>24</v>
       </c>
       <c r="N16" s="6">
-        <f>M16-SUM(N2:N15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
       <c r="O16" s="6">
-        <f>N16-SUM(O2:O15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
       <c r="P16" s="6">
-        <f>O16-SUM(P2:P15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="Q16" s="6">
-        <f>P16-SUM(Q2:Q15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="R16" s="6">
-        <f>Q16-SUM(R2:R15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="S16" s="6">
-        <f>R16-SUM(S2:S15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>11</v>
       </c>
       <c r="T16" s="6">
-        <f>S16-SUM(T2:T15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="U16" s="6">
-        <f>T16-SUM(U2:U15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="V16" s="6">
-        <f>U16-SUM(V2:V15)</f>
-        <v>40.5</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="W16" s="1"/>
     </row>
@@ -3050,86 +3094,86 @@
       </c>
       <c r="B17" s="8">
         <f>SUM(B2:B15)</f>
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="C17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>55.1</v>
+        <f t="shared" ref="C17:V17" si="1">$B$17-(($B$17/20)*(COLUMN()-2))</f>
+        <v>45.6</v>
       </c>
       <c r="D17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>52.2</v>
+        <f t="shared" si="1"/>
+        <v>43.2</v>
       </c>
       <c r="E17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>49.3</v>
+        <f t="shared" si="1"/>
+        <v>40.799999999999997</v>
       </c>
       <c r="F17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>46.4</v>
+        <f t="shared" si="1"/>
+        <v>38.4</v>
       </c>
       <c r="G17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>43.5</v>
+        <f t="shared" si="1"/>
+        <v>36</v>
       </c>
       <c r="H17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>40.6</v>
+        <f t="shared" si="1"/>
+        <v>33.6</v>
       </c>
       <c r="I17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>37.700000000000003</v>
+        <f t="shared" si="1"/>
+        <v>31.2</v>
       </c>
       <c r="J17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>34.799999999999997</v>
+        <f t="shared" si="1"/>
+        <v>28.8</v>
       </c>
       <c r="K17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>31.900000000000002</v>
+        <f t="shared" si="1"/>
+        <v>26.400000000000002</v>
       </c>
       <c r="L17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>29</v>
+        <f t="shared" si="1"/>
+        <v>24</v>
       </c>
       <c r="M17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>26.1</v>
+        <f t="shared" si="1"/>
+        <v>21.6</v>
       </c>
       <c r="N17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>23.200000000000003</v>
+        <f t="shared" si="1"/>
+        <v>19.200000000000003</v>
       </c>
       <c r="O17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>20.300000000000004</v>
+        <f t="shared" si="1"/>
+        <v>16.8</v>
       </c>
       <c r="P17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>17.399999999999999</v>
+        <f t="shared" si="1"/>
+        <v>14.399999999999999</v>
       </c>
       <c r="Q17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>14.5</v>
+        <f t="shared" si="1"/>
+        <v>12</v>
       </c>
       <c r="R17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>11.600000000000001</v>
+        <f t="shared" si="1"/>
+        <v>9.6000000000000014</v>
       </c>
       <c r="S17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>8.7000000000000028</v>
+        <f t="shared" si="1"/>
+        <v>7.2000000000000028</v>
       </c>
       <c r="T17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>5.8000000000000043</v>
+        <f t="shared" si="1"/>
+        <v>4.8000000000000043</v>
       </c>
       <c r="U17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>2.8999999999999986</v>
+        <f t="shared" si="1"/>
+        <v>2.3999999999999986</v>
       </c>
       <c r="V17" s="7">
-        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W17" s="1"/>

</xml_diff>